<commit_message>
feat: review spreadsheet codes and unify Excel output
</commit_message>
<xml_diff>
--- a/src/assets/store-order-template.xlsx
+++ b/src/assets/store-order-template.xlsx
@@ -1670,12 +1670,14 @@
       <x:c r="D6" s="90"/>
       <x:c r="E6" s="90"/>
     </x:row>
-    <x:row r="7" ht="32" customHeight="1">
+    <x:row r="7" ht="40" customHeight="1">
       <x:c r="A7" s="89" t="str">
         <x:v>2. Add products</x:v>
       </x:c>
-      <x:c r="B7" s="90" t="str">
-        <x:v>Use Orders rows 7–26. Keep row 5 markers. Fill Group to include a row; leave it blank to skip. Reuse a Group ID for related variants.</x:v>
+      <x:c r="B7" s="90" t="inlineStr">
+        <x:is>
+          <x:t>Use Orders rows 7–26. Keep row 5 markers. Fill Group to include a row; blank skips it. Equal Group values share one product base, even with different titles or separated rows.</x:t>
+        </x:is>
       </x:c>
       <x:c r="C7" s="90"/>
       <x:c r="D7" s="90"/>
@@ -1703,12 +1705,16 @@
       <x:c r="D9" s="90"/>
       <x:c r="E9" s="90"/>
     </x:row>
-    <x:row r="10" ht="32" customHeight="1">
-      <x:c r="A10" s="89" t="str">
-        <x:v>5. Save and review</x:v>
-      </x:c>
-      <x:c r="B10" s="90" t="str">
-        <x:v>Save in Excel or WPS before importing. Choose Orders, confirm the purchase date, review pictures, quantities and totals, then import.</x:v>
+    <x:row r="10" ht="44" customHeight="1">
+      <x:c r="A10" s="89" t="inlineStr">
+        <x:is>
+          <x:t>5. Save and review</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B10" s="90" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Save in Excel or WPS. Review the purchase date, photos, quantities and total, then choose Review products and codes. Edit details and endings before Import and assign codes.</x:t>
+        </x:is>
       </x:c>
       <x:c r="C10" s="90"/>
       <x:c r="D10" s="90"/>
@@ -1877,7 +1883,7 @@
         <x:v>Default formula: price × qty, rounded to cents. Import review detects a supplied amount that does not reconcile.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="38" customHeight="1">
+    <x:row r="22" ht="54" customHeight="1">
       <x:c r="A22" s="104" t="str">
         <x:v>group</x:v>
       </x:c>
@@ -1890,11 +1896,13 @@
       <x:c r="D22" s="107" t="str">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E22" s="98" t="str">
-        <x:v>Same ID joins related rows, even when they are separated. Blank group skips the whole row. IDs never assign a CE product code.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="38" customHeight="1">
+      <x:c r="E22" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Equal values share one editable product base, even across separated rows or different titles. Blank skips the row. A value such as 12 never assigns CE digits 0012.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="62" customHeight="1">
       <x:c r="A23" s="104" t="str">
         <x:v>var</x:v>
       </x:c>
@@ -1907,8 +1915,10 @@
       <x:c r="D23" s="107" t="str">
         <x:v>A / B / AB / ABS</x:v>
       </x:c>
-      <x:c r="E23" s="98" t="str">
-        <x:v>Use A and B for separate rows. AB means combined totals requiring manual allocation; ABS means A+B in size S.</x:v>
+      <x:c r="E23" s="98" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">A nonblank var is the complete suggested ending: a means A, s means size S, and as means AS. Description measurements do not add extra size endings. AB needs a reviewed quantity split; ABS means A+B in S. Blank var keeps normal suggestions.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="24" ht="38" customHeight="1">
@@ -2029,7 +2039,7 @@
       <x:c r="D31" s="10"/>
       <x:c r="E31" s="10"/>
     </x:row>
-    <x:row r="32" ht="38" customHeight="1">
+    <x:row r="32" ht="46" customHeight="1">
       <x:c r="A32" s="97" t="str">
         <x:v>One row per variant</x:v>
       </x:c>
@@ -2042,11 +2052,13 @@
       <x:c r="D32" s="97" t="str">
         <x:v>20 and 30 pieces</x:v>
       </x:c>
-      <x:c r="E32" s="97" t="str">
-        <x:v>Two product rows use the same group and each row has its own cartons, quantities, pictures and price.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="38" customHeight="1">
+      <x:c r="E32" s="97" t="inlineStr">
+        <x:is>
+          <x:t>Both rows share one editable product base, even if titles differ. Each source row keeps its own pictures, cartons, quantity and price.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="46" customHeight="1">
       <x:c r="A33" s="98" t="str">
         <x:v>Combined variants</x:v>
       </x:c>
@@ -2059,11 +2071,13 @@
       <x:c r="D33" s="98" t="str">
         <x:v>40 combined pieces</x:v>
       </x:c>
-      <x:c r="E33" s="98" t="str">
-        <x:v>One row covers A and B together. Enter the real per-variant quantities during review. The importer never divides them equally for you.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="38" customHeight="1">
+      <x:c r="E33" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Enter actual positive A/B quantities summing to 40. Preserve the source amount. The source cartons are retained once, never copied to each variant.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="54" customHeight="1">
       <x:c r="A34" s="98" t="str">
         <x:v>Models and sizes</x:v>
       </x:c>
@@ -2076,8 +2090,10 @@
       <x:c r="D34" s="98" t="str">
         <x:v>A+B by size</x:v>
       </x:c>
-      <x:c r="E34" s="98" t="str">
-        <x:v>ABS means A+B in size S; ABM and ABL use sizes M and L. Each combined row needs a reviewed split.</x:v>
+      <x:c r="E34" s="98" t="inlineStr">
+        <x:is>
+          <x:t>abs, abm and abl mean A+B in S, M and L. Review each combined row’s quantities, then variant/size endings. Unknown sizes block final import.</x:t>
+        </x:is>
       </x:c>
     </x:row>
     <x:row r="35" ht="38" customHeight="1">
@@ -2104,9 +2120,11 @@
       <x:c r="D36" s="2"/>
       <x:c r="E36" s="2"/>
     </x:row>
-    <x:row r="37" ht="28" customHeight="1">
-      <x:c r="A37" s="110" t="str">
-        <x:v>Missing pictures, conflicting quantities or prices, and formula errors must be corrected before import.</x:v>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="110" t="inlineStr">
+        <x:is>
+          <x:t>Missing pictures, incorrect totals, unresolved sizes and invalid or conflicting codes block final import. Correct each issue before confirming.</x:t>
+        </x:is>
       </x:c>
       <x:c r="B37" s="110"/>
       <x:c r="C37" s="110"/>
@@ -2135,6 +2153,520 @@
       <x:c r="C40" s="2"/>
       <x:c r="D40" s="2"/>
       <x:c r="E40" s="2"/>
+    </x:row>
+    <x:row r="41" ht="25" customHeight="1">
+      <x:c r="A41" s="10" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Review products and codes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B41" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="C41" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D41" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E41" s="10" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="40" customHeight="1">
+      <x:c r="A42" s="89" t="inlineStr">
+        <x:is>
+          <x:t>1. Check workbook</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B42" s="90" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Confirm the purchase date and check photos, quantities, combined-variant allocations and invoice total. Review products and codes becomes available after these checks.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C42" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D42" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E42" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="40" customHeight="1">
+      <x:c r="A43" s="89" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">2. Review products</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B43" s="90" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Review products and codes opens editable details and proposals. It does not save an order, photos or preparation and does not reserve codes.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C43" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D43" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E43" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="40" customHeight="1">
+      <x:c r="A44" s="89" t="inlineStr">
+        <x:is>
+          <x:t>3. Edit group base</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B44" s="90" t="inlineStr">
+        <x:is>
+          <x:t>Edit one CE base for the whole source group. Equal group values stay together regardless of title or row position; group text is not assigned CE digits.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C44" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D44" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E44" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="40" customHeight="1">
+      <x:c r="A45" s="89" t="inlineStr">
+        <x:is>
+          <x:t>4. Edit endings</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B45" s="90" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Review each variant ending and size ending. Full barcodes update as you edit. Nonblank var declarations are complete endings. Resolve unknown inferred sizes or choose Do not add size endings; physical measurements stay in descriptions.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C45" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D45" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E45" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="40" customHeight="1">
+      <x:c r="A46" s="89" t="inlineStr">
+        <x:is>
+          <x:t>5. Confirm import</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B46" s="90" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Import and assign codes revalidates the current library and saves the order, photos, authored details, preparation, code assignments and source carton facts together. A failure saves none of them.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C46" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D46" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E46" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="0" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="B47" s="0" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="C47" s="0" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D47" s="0" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E47" s="0" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="28" customHeight="1">
+      <x:c r="A48" s="93" t="inlineStr">
+        <x:is>
+          <x:t>Example</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B48" s="93" t="inlineStr">
+        <x:is>
+          <x:t>Source group</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C48" s="93" t="inlineStr">
+        <x:is>
+          <x:t>var / size</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D48" s="93" t="inlineStr">
+        <x:is>
+          <x:t>Proposed result</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E48" s="93" t="inlineStr">
+        <x:is>
+          <x:t>Review meaning</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="62" customHeight="1">
+      <x:c r="A49" s="97" t="inlineStr">
+        <x:is>
+          <x:t>Same group</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B49" s="97" t="inlineStr">
+        <x:is>
+          <x:t>tray · rows 7 and 10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C49" s="97" t="inlineStr">
+        <x:is>
+          <x:t>A, then B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D49" s="97" t="inlineStr">
+        <x:is>
+          <x:t>CE26100101A
+CE26100101B</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E49" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Both share CE26100101, even with different titles. A base edit updates both. The literal group tray never sets CE digits. A/B declarations remain A/B even when descriptions contain different measurements.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="62" customHeight="1">
+      <x:c r="A50" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Combined row</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B50" s="98" t="inlineStr">
+        <x:is>
+          <x:t>mix · one row</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C50" s="98" t="inlineStr">
+        <x:is>
+          <x:t>abcd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D50" s="98" t="inlineStr">
+        <x:is>
+          <x:t>40 pieces: 7 / 11 / 9 / 13</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E50" s="98" t="inlineStr">
+        <x:is>
+          <x:t>The actual split sums to 40 and preserves the row amount. Confirm its source cartons once; do not multiply cartons by four.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="62" customHeight="1">
+      <x:c r="A51" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Models and sizes</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B51" s="98" t="inlineStr">
+        <x:is>
+          <x:t>shirt</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C51" s="98" t="inlineStr">
+        <x:is>
+          <x:t>abs</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D51" s="98" t="inlineStr">
+        <x:is>
+          <x:t>A + S / B + S</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E51" s="98" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Allocate the real A/B quantities in size S. Review both endings and full barcodes. Do not add size endings is an explicit coding choice, not a claim that physical sizes are equal.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="62" customHeight="1">
+      <x:c r="A52" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Valid ownership</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B52" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Purchase: 2026-10</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C52" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Known supplier</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D52" s="98" t="inlineStr">
+        <x:is>
+          <x:t>CE26100101</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E52" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Illustrative October 2026 base only. Actual proposals must use the purchase month and known supplier and respect current assignments and immutable shipment history.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="62" customHeight="1">
+      <x:c r="A53" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Return or reset</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B53" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Back / Cancel</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C53" s="98" t="inlineStr">
+        <x:is>
+          <x:t>Reset to suggested</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D53" s="98" t="inlineStr">
+        <x:is>
+          <x:t>No reservation</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E53" s="98" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Back returns to workbook checks; Cancel exits without saving; Reset to suggested restores proposals while preserving authored details. A conflict before final save blocks the whole import.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="40" customHeight="1">
+      <x:c r="A54" s="89" t="inlineStr">
+        <x:is>
+          <x:t>Source facts</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B54" s="90" t="inlineStr">
+        <x:is>
+          <x:t>Code edits retain original photos, marked descriptions, purchase quantities, prices and totals. Source carton facts remain separate from barcode endings and later physical-packing decisions.</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C54" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="D54" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+      <x:c r="E54" s="90" t="inlineStr">
+        <x:is>
+          <x:t/>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="28" customHeight="1">
+      <x:c r="A56" s="93" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Scope</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B56" s="93" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Control</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C56" s="93" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Spanish name</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D56" s="93" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Chinese category</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E56" s="93" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Material and exceptions</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="62" customHeight="1">
+      <x:c r="A57" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Entire order</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B57" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Edit order details</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C57" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">All groups</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D57" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">All groups; each carton mark keeps its group value</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E57" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">All variants and source rows in the purchase. Keep custom values preserves manual exceptions and deliberate blanks by default.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="62" customHeight="1">
+      <x:c r="A58" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">CE product group</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B58" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Edit group details</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C58" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared base name and variant exceptions</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D58" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">One shared carton-mark category</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E58" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">All variants and source rows in one CE group. Mixed materials remain visible.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="62" customHeight="1">
+      <x:c r="A59" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Individual variant</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B59" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Edit variant details</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C59" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">One barcode identity</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D59" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Shared group value; use Edit group category</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E59" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">The variant's source rows. A shared Spanish name affects every row with that barcode, without combining quantities or prices.</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="62" customHeight="1">
+      <x:c r="A60" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Apply or cancel</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B60" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Choose fields before Apply</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C60" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Untouched fields stay unchanged</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D60" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Replace all values replaces custom exceptions explicitly</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E60" s="97" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Review affected counts. Cancel changes nothing. Controls also appear in Orders. Correct existing codes through group size handling; do not reimport a purchase to repair its codes.</x:t>
+        </x:is>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2144,6 +2676,12 @@
     <x:mergeCell ref="B9:E9"/>
     <x:mergeCell ref="B10:E10"/>
     <x:mergeCell ref="B11:E11"/>
+    <x:mergeCell ref="B42:E42"/>
+    <x:mergeCell ref="B43:E43"/>
+    <x:mergeCell ref="B44:E44"/>
+    <x:mergeCell ref="B45:E45"/>
+    <x:mergeCell ref="B46:E46"/>
+    <x:mergeCell ref="B54:E54"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>